<commit_message>
Refactor payroll seeding and enhance email notifications
This update modifies the payroll seeding process for 2025 by truncating existing data instead of deleting it, improving efficiency. Additionally, it introduces email notifications for claim and leave status updates, as well as for sending payslips and EA forms, enhancing user communication. The email templates for claims and EA forms have also been added, ensuring a consistent and professional format for notifications.
</commit_message>
<xml_diff>
--- a/docs/data/Payroll_Statutory_2025/Mohammad Amier Akram bin Mohd Zaki.xlsx
+++ b/docs/data/Payroll_Statutory_2025/Mohammad Amier Akram bin Mohd Zaki.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haziq\Averroes Data Science\Company\Velarix Technology Sdn Bhd\HR\Payslip\Statutory 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{29F8CA02-7E54-4C30-9D8C-C82E7A38014C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019B0F13-19FE-43FC-9CE0-B38BAA71731D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B1B849BC-E9C4-4F7B-967D-F42DB3982308}"/>
   </bookViews>
@@ -244,50 +244,50 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,853 +596,853 @@
   <dimension ref="A1:R14"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="8.88671875" style="8"/>
-    <col min="4" max="4" width="10.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.88671875" style="8"/>
-    <col min="8" max="8" width="11.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="8.88671875" style="8"/>
-    <col min="12" max="12" width="11.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="8.88671875" style="8"/>
-    <col min="16" max="16" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.88671875" style="8"/>
+    <col min="1" max="3" width="8.88671875" style="5"/>
+    <col min="4" max="4" width="10.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.88671875" style="5"/>
+    <col min="8" max="8" width="11.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="8.88671875" style="5"/>
+    <col min="12" max="12" width="11.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="8.88671875" style="5"/>
+    <col min="16" max="16" width="13.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1" t="s">
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1" t="s">
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1" t="s">
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
     </row>
-    <row r="2" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="5" t="s">
+    <row r="2" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="Q2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="R2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>2025</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>8500</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <f>C3-SUM(E3:H3)</f>
         <v>6914.15</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="4">
         <v>935</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="4">
         <v>29.75</v>
       </c>
-      <c r="G3" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H3" s="7">
+      <c r="G3" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H3" s="4">
         <v>609.20000000000005</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="4">
         <f>SUM(E3)</f>
         <v>935</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="4">
         <f t="shared" ref="J3:L3" si="0">SUM(F3)</f>
         <v>29.75</v>
       </c>
-      <c r="K3" s="7">
+      <c r="K3" s="4">
         <f t="shared" si="0"/>
         <v>11.9</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="4">
         <f t="shared" si="0"/>
         <v>609.20000000000005</v>
       </c>
-      <c r="M3" s="7">
+      <c r="M3" s="4">
         <v>1105</v>
       </c>
-      <c r="N3" s="7">
+      <c r="N3" s="4">
         <v>104.15</v>
       </c>
-      <c r="O3" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P3" s="7">
+      <c r="O3" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P3" s="4">
         <f>SUM(M3)</f>
         <v>1105</v>
       </c>
-      <c r="Q3" s="7">
+      <c r="Q3" s="4">
         <f>SUM(N3)</f>
         <v>104.15</v>
       </c>
-      <c r="R3" s="7">
+      <c r="R3" s="4">
         <f>SUM(O3)</f>
         <v>11.9</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
+      <c r="A4" s="3">
         <v>2025</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>8500</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <f t="shared" ref="D4:D13" si="1">C4-SUM(E4:H4)</f>
         <v>6914.15</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="4">
         <v>935</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="4">
         <v>29.75</v>
       </c>
-      <c r="G4" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H4" s="7">
+      <c r="G4" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H4" s="4">
         <v>609.20000000000005</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="4">
         <f>SUM(I3,E4)</f>
         <v>1870</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="4">
         <f t="shared" ref="J4:L13" si="2">SUM(J3,F4)</f>
         <v>59.5</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="4">
         <f t="shared" si="2"/>
         <v>23.8</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="4">
         <f t="shared" si="2"/>
         <v>1218.4000000000001</v>
       </c>
-      <c r="M4" s="7">
+      <c r="M4" s="4">
         <v>1105</v>
       </c>
-      <c r="N4" s="7">
+      <c r="N4" s="4">
         <v>104.15</v>
       </c>
-      <c r="O4" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P4" s="7">
+      <c r="O4" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P4" s="4">
         <f>SUM(P3,M4)</f>
         <v>2210</v>
       </c>
-      <c r="Q4" s="7">
+      <c r="Q4" s="4">
         <f>SUM(Q3,N4)</f>
         <v>208.3</v>
       </c>
-      <c r="R4" s="7">
+      <c r="R4" s="4">
         <f>SUM(R3,O4)</f>
         <v>23.8</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>2025</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>8500</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <f t="shared" si="1"/>
-        <v>6914.15</v>
-      </c>
-      <c r="E5" s="7">
+        <v>6914.2</v>
+      </c>
+      <c r="E5" s="4">
         <v>935</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="4">
         <v>29.75</v>
       </c>
-      <c r="G5" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H5" s="7">
-        <v>609.20000000000005</v>
-      </c>
-      <c r="I5" s="7">
+      <c r="G5" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H5" s="4">
+        <v>609.15</v>
+      </c>
+      <c r="I5" s="4">
         <f t="shared" ref="I5:I13" si="3">SUM(I4,E5)</f>
         <v>2805</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="4">
         <f t="shared" si="2"/>
         <v>89.25</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="4">
         <f t="shared" si="2"/>
         <v>35.700000000000003</v>
       </c>
-      <c r="L5" s="7">
-        <f t="shared" si="2"/>
-        <v>1827.6000000000001</v>
-      </c>
-      <c r="M5" s="7">
+      <c r="L5" s="4">
+        <f t="shared" si="2"/>
+        <v>1827.5500000000002</v>
+      </c>
+      <c r="M5" s="4">
         <v>1105</v>
       </c>
-      <c r="N5" s="7">
+      <c r="N5" s="4">
         <v>104.15</v>
       </c>
-      <c r="O5" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P5" s="7">
+      <c r="O5" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P5" s="4">
         <f t="shared" ref="P5:R13" si="4">SUM(P4,M5)</f>
         <v>3315</v>
       </c>
-      <c r="Q5" s="7">
+      <c r="Q5" s="4">
         <f t="shared" si="4"/>
         <v>312.45000000000005</v>
       </c>
-      <c r="R5" s="7">
+      <c r="R5" s="4">
         <f t="shared" si="4"/>
         <v>35.700000000000003</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
+      <c r="A6" s="3">
         <v>2025</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="3">
         <v>8500</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <f t="shared" si="1"/>
-        <v>6914.15</v>
-      </c>
-      <c r="E6" s="7">
+        <v>7009.2</v>
+      </c>
+      <c r="E6" s="4">
         <v>935</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="4">
         <v>29.75</v>
       </c>
-      <c r="G6" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H6" s="7">
-        <v>609.20000000000005</v>
-      </c>
-      <c r="I6" s="7">
+      <c r="G6" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H6" s="4">
+        <v>514.15</v>
+      </c>
+      <c r="I6" s="4">
         <f t="shared" si="3"/>
         <v>3740</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="4">
         <f t="shared" si="2"/>
         <v>119</v>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="4">
         <f t="shared" si="2"/>
         <v>47.6</v>
       </c>
-      <c r="L6" s="7">
-        <f t="shared" si="2"/>
-        <v>2436.8000000000002</v>
-      </c>
-      <c r="M6" s="7">
+      <c r="L6" s="4">
+        <f t="shared" si="2"/>
+        <v>2341.7000000000003</v>
+      </c>
+      <c r="M6" s="4">
         <v>1105</v>
       </c>
-      <c r="N6" s="7">
+      <c r="N6" s="4">
         <v>104.15</v>
       </c>
-      <c r="O6" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P6" s="7">
+      <c r="O6" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P6" s="4">
         <f t="shared" si="4"/>
         <v>4420</v>
       </c>
-      <c r="Q6" s="7">
+      <c r="Q6" s="4">
         <f t="shared" si="4"/>
         <v>416.6</v>
       </c>
-      <c r="R6" s="7">
+      <c r="R6" s="4">
         <f t="shared" si="4"/>
         <v>47.6</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
+      <c r="A7" s="3">
         <v>2025</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="3">
         <v>8500</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <f t="shared" si="1"/>
-        <v>6914.15</v>
-      </c>
-      <c r="E7" s="7">
+        <v>7009.2</v>
+      </c>
+      <c r="E7" s="4">
         <v>935</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="4">
         <v>29.75</v>
       </c>
-      <c r="G7" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H7" s="7">
-        <v>609.20000000000005</v>
-      </c>
-      <c r="I7" s="7">
+      <c r="G7" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H7" s="4">
+        <v>514.15</v>
+      </c>
+      <c r="I7" s="4">
         <f t="shared" si="3"/>
         <v>4675</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="4">
         <f t="shared" si="2"/>
         <v>148.75</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="4">
         <f t="shared" si="2"/>
         <v>59.5</v>
       </c>
-      <c r="L7" s="7">
-        <f t="shared" si="2"/>
-        <v>3046</v>
-      </c>
-      <c r="M7" s="7">
+      <c r="L7" s="4">
+        <f t="shared" si="2"/>
+        <v>2855.8500000000004</v>
+      </c>
+      <c r="M7" s="4">
         <v>1105</v>
       </c>
-      <c r="N7" s="7">
+      <c r="N7" s="4">
         <v>104.15</v>
       </c>
-      <c r="O7" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P7" s="7">
+      <c r="O7" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P7" s="4">
         <f t="shared" si="4"/>
         <v>5525</v>
       </c>
-      <c r="Q7" s="7">
+      <c r="Q7" s="4">
         <f t="shared" si="4"/>
         <v>520.75</v>
       </c>
-      <c r="R7" s="7">
+      <c r="R7" s="4">
         <f t="shared" si="4"/>
         <v>59.5</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+      <c r="A8" s="3">
         <v>2025</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="3">
         <v>8500</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <f t="shared" si="1"/>
-        <v>6914.15</v>
-      </c>
-      <c r="E8" s="7">
+        <v>7009.2</v>
+      </c>
+      <c r="E8" s="4">
         <v>935</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="4">
         <v>29.75</v>
       </c>
-      <c r="G8" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H8" s="7">
-        <v>609.20000000000005</v>
-      </c>
-      <c r="I8" s="7">
+      <c r="G8" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H8" s="4">
+        <v>514.15</v>
+      </c>
+      <c r="I8" s="4">
         <f t="shared" si="3"/>
         <v>5610</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="4">
         <f t="shared" si="2"/>
         <v>178.5</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="4">
         <f t="shared" si="2"/>
         <v>71.400000000000006</v>
       </c>
-      <c r="L8" s="7">
-        <f t="shared" si="2"/>
-        <v>3655.2</v>
-      </c>
-      <c r="M8" s="7">
+      <c r="L8" s="4">
+        <f t="shared" si="2"/>
+        <v>3370.0000000000005</v>
+      </c>
+      <c r="M8" s="4">
         <v>1105</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="4">
         <v>104.15</v>
       </c>
-      <c r="O8" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P8" s="7">
+      <c r="O8" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P8" s="4">
         <f t="shared" si="4"/>
         <v>6630</v>
       </c>
-      <c r="Q8" s="7">
+      <c r="Q8" s="4">
         <f t="shared" si="4"/>
         <v>624.9</v>
       </c>
-      <c r="R8" s="7">
+      <c r="R8" s="4">
         <f t="shared" si="4"/>
         <v>71.400000000000006</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+      <c r="A9" s="3">
         <v>2025</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>8500</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <f t="shared" si="1"/>
         <v>7009.15</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="4">
         <v>935</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="4">
         <v>29.75</v>
       </c>
-      <c r="G9" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H9" s="7">
+      <c r="G9" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H9" s="4">
         <v>514.20000000000005</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="4">
         <f t="shared" si="3"/>
         <v>6545</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="4">
         <f t="shared" si="2"/>
         <v>208.25</v>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="4">
         <f t="shared" si="2"/>
         <v>83.300000000000011</v>
       </c>
-      <c r="L9" s="7">
-        <f t="shared" si="2"/>
-        <v>4169.3999999999996</v>
-      </c>
-      <c r="M9" s="7">
+      <c r="L9" s="4">
+        <f t="shared" si="2"/>
+        <v>3884.2000000000007</v>
+      </c>
+      <c r="M9" s="4">
         <v>1105</v>
       </c>
-      <c r="N9" s="7">
+      <c r="N9" s="4">
         <v>104.15</v>
       </c>
-      <c r="O9" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P9" s="7">
+      <c r="O9" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P9" s="4">
         <f t="shared" si="4"/>
         <v>7735</v>
       </c>
-      <c r="Q9" s="7">
+      <c r="Q9" s="4">
         <f t="shared" si="4"/>
         <v>729.05</v>
       </c>
-      <c r="R9" s="7">
+      <c r="R9" s="4">
         <f t="shared" si="4"/>
         <v>83.300000000000011</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+      <c r="A10" s="3">
         <v>2025</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>8500</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <f t="shared" si="1"/>
         <v>7009.2</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="4">
         <v>935</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="4">
         <v>29.75</v>
       </c>
-      <c r="G10" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H10" s="7">
+      <c r="G10" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H10" s="4">
         <v>514.15</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="4">
         <f t="shared" si="3"/>
         <v>7480</v>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="4">
         <f t="shared" si="2"/>
         <v>238</v>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="4">
         <f t="shared" si="2"/>
         <v>95.200000000000017</v>
       </c>
-      <c r="L10" s="7">
-        <f t="shared" si="2"/>
-        <v>4683.5499999999993</v>
-      </c>
-      <c r="M10" s="7">
+      <c r="L10" s="4">
+        <f t="shared" si="2"/>
+        <v>4398.3500000000004</v>
+      </c>
+      <c r="M10" s="4">
         <v>1105</v>
       </c>
-      <c r="N10" s="7">
+      <c r="N10" s="4">
         <v>104.15</v>
       </c>
-      <c r="O10" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P10" s="7">
+      <c r="O10" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P10" s="4">
         <f t="shared" si="4"/>
         <v>8840</v>
       </c>
-      <c r="Q10" s="7">
+      <c r="Q10" s="4">
         <f t="shared" si="4"/>
         <v>833.19999999999993</v>
       </c>
-      <c r="R10" s="7">
+      <c r="R10" s="4">
         <f t="shared" si="4"/>
         <v>95.200000000000017</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+      <c r="A11" s="3">
         <v>2025</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>8500</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <f t="shared" si="1"/>
         <v>7009.2</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="4">
         <v>935</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="4">
         <v>29.75</v>
       </c>
-      <c r="G11" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H11" s="7">
+      <c r="G11" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H11" s="4">
         <v>514.15</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="4">
         <f t="shared" si="3"/>
         <v>8415</v>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="4">
         <f t="shared" si="2"/>
         <v>267.75</v>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="4">
         <f t="shared" si="2"/>
         <v>107.10000000000002</v>
       </c>
-      <c r="L11" s="7">
-        <f t="shared" si="2"/>
-        <v>5197.6999999999989</v>
-      </c>
-      <c r="M11" s="7">
+      <c r="L11" s="4">
+        <f t="shared" si="2"/>
+        <v>4912.5</v>
+      </c>
+      <c r="M11" s="4">
         <v>1105</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="4">
         <v>104.15</v>
       </c>
-      <c r="O11" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P11" s="7">
+      <c r="O11" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P11" s="4">
         <f t="shared" si="4"/>
         <v>9945</v>
       </c>
-      <c r="Q11" s="7">
+      <c r="Q11" s="4">
         <f t="shared" si="4"/>
         <v>937.34999999999991</v>
       </c>
-      <c r="R11" s="7">
+      <c r="R11" s="4">
         <f t="shared" si="4"/>
         <v>107.10000000000002</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+      <c r="A12" s="3">
         <v>2025</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>8500</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <f t="shared" si="1"/>
         <v>7009.2</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="4">
         <v>935</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="4">
         <v>29.75</v>
       </c>
-      <c r="G12" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H12" s="7">
+      <c r="G12" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H12" s="4">
         <v>514.15</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="4">
         <f t="shared" si="3"/>
         <v>9350</v>
       </c>
-      <c r="J12" s="7">
+      <c r="J12" s="4">
         <f t="shared" si="2"/>
         <v>297.5</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="4">
         <f t="shared" si="2"/>
         <v>119.00000000000003</v>
       </c>
-      <c r="L12" s="7">
-        <f t="shared" si="2"/>
-        <v>5711.8499999999985</v>
-      </c>
-      <c r="M12" s="7">
+      <c r="L12" s="4">
+        <f t="shared" si="2"/>
+        <v>5426.65</v>
+      </c>
+      <c r="M12" s="4">
         <v>1105</v>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="4">
         <v>104.15</v>
       </c>
-      <c r="O12" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P12" s="7">
+      <c r="O12" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P12" s="4">
         <f t="shared" si="4"/>
         <v>11050</v>
       </c>
-      <c r="Q12" s="7">
+      <c r="Q12" s="4">
         <f t="shared" si="4"/>
         <v>1041.5</v>
       </c>
-      <c r="R12" s="7">
+      <c r="R12" s="4">
         <f t="shared" si="4"/>
         <v>119.00000000000003</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
+      <c r="A13" s="3">
         <v>2025</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="3">
         <v>9500</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="3">
         <f t="shared" si="1"/>
         <v>7709.2</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="4">
         <v>1045</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="4">
         <v>29.75</v>
       </c>
-      <c r="G13" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="H13" s="7">
+      <c r="G13" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="H13" s="4">
         <v>704.15</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="4">
         <f t="shared" si="3"/>
         <v>10395</v>
       </c>
-      <c r="J13" s="7">
+      <c r="J13" s="4">
         <f t="shared" si="2"/>
         <v>327.25</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="4">
         <f t="shared" si="2"/>
         <v>130.90000000000003</v>
       </c>
-      <c r="L13" s="7">
-        <f t="shared" si="2"/>
-        <v>6415.9999999999982</v>
-      </c>
-      <c r="M13" s="7">
+      <c r="L13" s="4">
+        <f t="shared" si="2"/>
+        <v>6130.7999999999993</v>
+      </c>
+      <c r="M13" s="4">
         <v>1235</v>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="4">
         <v>104.15</v>
       </c>
-      <c r="O13" s="7">
-        <v>11.9</v>
-      </c>
-      <c r="P13" s="7">
+      <c r="O13" s="4">
+        <v>11.9</v>
+      </c>
+      <c r="P13" s="4">
         <f t="shared" si="4"/>
         <v>12285</v>
       </c>
-      <c r="Q13" s="7">
+      <c r="Q13" s="4">
         <f t="shared" si="4"/>
         <v>1145.6500000000001</v>
       </c>
-      <c r="R13" s="7">
+      <c r="R13" s="4">
         <f t="shared" si="4"/>
         <v>130.90000000000003</v>
       </c>
     </row>
-    <row r="14" spans="1:18" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11">
+      <c r="B14" s="11"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6">
         <f>SUM(D3:D13)</f>
-        <v>77230.849999999991</v>
-      </c>
-      <c r="E14" s="12">
+        <v>77516.049999999988</v>
+      </c>
+      <c r="E14" s="7">
         <f>SUM(E3:E13)</f>
         <v>10395</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="7">
         <f>SUM(F3:F13)</f>
         <v>327.25</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="7">
         <f>SUM(G3:G13)</f>
         <v>130.90000000000003</v>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="7">
         <f>SUM(H3:H13)</f>
-        <v>6415.9999999999982</v>
-      </c>
-      <c r="I14" s="13"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="12">
+        <v>6130.7999999999993</v>
+      </c>
+      <c r="I14" s="12"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="14"/>
+      <c r="M14" s="7">
         <f>SUM(M3:M13)</f>
         <v>12285</v>
       </c>
-      <c r="N14" s="12">
+      <c r="N14" s="7">
         <f>SUM(N3:N13)</f>
         <v>1145.6500000000001</v>
       </c>
-      <c r="O14" s="12">
+      <c r="O14" s="7">
         <f>SUM(O3:O13)</f>
         <v>130.90000000000003</v>
       </c>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="14"/>
-      <c r="R14" s="15"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="13"/>
+      <c r="R14" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>